<commit_message>
mod: latest updates according to Github issues
</commit_message>
<xml_diff>
--- a/Symbols_UpdateReferenceID.xlsx
+++ b/Symbols_UpdateReferenceID.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\DISCDEXPI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mso\Desktop\todo\discII\github\DISCDEXPI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF25E484-CEE5-43E7-8FEA-7AE7894E6738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{D5E47F2D-020A-4A1E-8973-8478EA58E23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="524" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="524" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Symbols" sheetId="1" r:id="rId1"/>
@@ -25,9 +25,9 @@
     <definedName name="RowEnd">Symbols!$B$1</definedName>
     <definedName name="RowStart">Symbols!$A$1</definedName>
     <definedName name="TR1970id">#REF!</definedName>
-    <definedName name="Z004id">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -55,27 +55,27 @@
   <commentList>
     <comment ref="C24" authorId="0" shapeId="0" xr:uid="{A32D579A-03F5-456F-BA00-67936BD401D0}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     MCC/VSD/THY/MCS
-Reply:
+Antwort:
     Must support signal connection</t>
       </text>
     </comment>
     <comment ref="C139" authorId="1" shapeId="0" xr:uid="{36C2758C-D037-4478-BDED-0DD258CAD031}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     No signal</t>
       </text>
     </comment>
     <comment ref="C140" authorId="2" shapeId="0" xr:uid="{FBC2CACE-2F03-4DAC-8894-89865648F172}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
     No Signal - in-line</t>
       </text>
     </comment>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="719">
   <si>
     <t>Description</t>
   </si>
@@ -2228,6 +2228,24 @@
   </si>
   <si>
     <t>Electric Gas Heater</t>
+  </si>
+  <si>
+    <t>ND0251</t>
+  </si>
+  <si>
+    <t>Nozzle Hose Connector</t>
+  </si>
+  <si>
+    <t>ND0252</t>
+  </si>
+  <si>
+    <t>Demisting Cyclone Part</t>
+  </si>
+  <si>
+    <t>ND0253</t>
+  </si>
+  <si>
+    <t>Vessel Insulation</t>
   </si>
 </sst>
 </file>
@@ -2348,7 +2366,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2372,10 +2390,12 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -2413,9 +2433,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2453,7 +2473,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2559,7 +2579,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2727,19 +2747,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C270"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C273"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="197.42578125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="197.44140625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="6"/>
       <c r="C1" s="4"/>
     </row>
-    <row r="2" spans="1:3" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>694</v>
       </c>
@@ -2750,7 +2770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>391</v>
       </c>
@@ -2761,7 +2781,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>352</v>
       </c>
@@ -2772,7 +2792,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
         <v>1</v>
       </c>
@@ -2783,7 +2803,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>347</v>
       </c>
@@ -2794,7 +2814,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>349</v>
       </c>
@@ -2805,7 +2825,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
         <v>351</v>
       </c>
@@ -2816,7 +2836,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
         <v>13</v>
       </c>
@@ -2827,7 +2847,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
         <v>14</v>
       </c>
@@ -2838,7 +2858,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
         <v>634</v>
       </c>
@@ -2849,7 +2869,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
         <v>635</v>
       </c>
@@ -2860,7 +2880,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
         <v>636</v>
       </c>
@@ -2871,7 +2891,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
         <v>637</v>
       </c>
@@ -2882,7 +2902,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="15" t="s">
         <v>18</v>
       </c>
@@ -2893,7 +2913,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="15" t="s">
         <v>46</v>
       </c>
@@ -2904,7 +2924,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="15" t="s">
         <v>399</v>
       </c>
@@ -2915,7 +2935,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
         <v>53</v>
       </c>
@@ -2926,7 +2946,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
         <v>236</v>
       </c>
@@ -2937,7 +2957,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
         <v>358</v>
       </c>
@@ -2948,7 +2968,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
         <v>296</v>
       </c>
@@ -2959,7 +2979,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
         <v>364</v>
       </c>
@@ -2970,7 +2990,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="15" t="s">
         <v>365</v>
       </c>
@@ -2981,7 +3001,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="15" t="s">
         <v>366</v>
       </c>
@@ -2992,7 +3012,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="15" t="s">
         <v>367</v>
       </c>
@@ -3003,7 +3023,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="15" t="s">
         <v>369</v>
       </c>
@@ -3014,7 +3034,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
         <v>370</v>
       </c>
@@ -3025,7 +3045,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
         <v>377</v>
       </c>
@@ -3036,7 +3056,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
         <v>380</v>
       </c>
@@ -3047,7 +3067,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
         <v>381</v>
       </c>
@@ -3058,7 +3078,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
         <v>383</v>
       </c>
@@ -3069,7 +3089,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
         <v>384</v>
       </c>
@@ -3080,7 +3100,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>386</v>
       </c>
@@ -3091,7 +3111,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
         <v>387</v>
       </c>
@@ -3102,7 +3122,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
         <v>404</v>
       </c>
@@ -3113,7 +3133,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="15" t="s">
         <v>388</v>
       </c>
@@ -3124,7 +3144,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="15" t="s">
         <v>405</v>
       </c>
@@ -3135,7 +3155,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
         <v>389</v>
       </c>
@@ -3146,7 +3166,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="15" t="s">
         <v>394</v>
       </c>
@@ -3157,7 +3177,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="15" t="s">
         <v>395</v>
       </c>
@@ -3168,7 +3188,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
         <v>638</v>
       </c>
@@ -3179,7 +3199,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="15" t="s">
         <v>639</v>
       </c>
@@ -3190,7 +3210,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
         <v>640</v>
       </c>
@@ -3201,7 +3221,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="15" t="s">
         <v>641</v>
       </c>
@@ -3212,7 +3232,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="15" t="s">
         <v>442</v>
       </c>
@@ -3223,7 +3243,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
         <v>444</v>
       </c>
@@ -3234,7 +3254,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="15" t="s">
         <v>445</v>
       </c>
@@ -3245,7 +3265,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="15" t="s">
         <v>447</v>
       </c>
@@ -3256,7 +3276,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="15" t="s">
         <v>449</v>
       </c>
@@ -3267,7 +3287,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="15" t="s">
         <v>453</v>
       </c>
@@ -3278,7 +3298,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="15" t="s">
         <v>455</v>
       </c>
@@ -3289,7 +3309,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="15" t="s">
         <v>457</v>
       </c>
@@ -3300,7 +3320,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="15" t="s">
         <v>459</v>
       </c>
@@ -3311,7 +3331,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>703</v>
       </c>
@@ -3322,7 +3342,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>704</v>
       </c>
@@ -3333,7 +3353,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>705</v>
       </c>
@@ -3344,7 +3364,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>706</v>
       </c>
@@ -3355,7 +3375,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>461</v>
       </c>
@@ -3366,7 +3386,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>462</v>
       </c>
@@ -3377,7 +3397,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>463</v>
       </c>
@@ -3388,7 +3408,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>464</v>
       </c>
@@ -3399,7 +3419,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>465</v>
       </c>
@@ -3410,7 +3430,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>466</v>
       </c>
@@ -3421,7 +3441,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>467</v>
       </c>
@@ -3432,7 +3452,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>468</v>
       </c>
@@ -3443,7 +3463,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>469</v>
       </c>
@@ -3454,7 +3474,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>470</v>
       </c>
@@ -3465,7 +3485,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>471</v>
       </c>
@@ -3476,7 +3496,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>472</v>
       </c>
@@ -3487,7 +3507,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>473</v>
       </c>
@@ -3498,7 +3518,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>474</v>
       </c>
@@ -3509,7 +3529,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>475</v>
       </c>
@@ -3520,7 +3540,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>476</v>
       </c>
@@ -3531,7 +3551,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>477</v>
       </c>
@@ -3542,7 +3562,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>478</v>
       </c>
@@ -3553,7 +3573,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>479</v>
       </c>
@@ -3564,7 +3584,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>480</v>
       </c>
@@ -3575,7 +3595,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>481</v>
       </c>
@@ -3586,7 +3606,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>482</v>
       </c>
@@ -3597,7 +3617,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>483</v>
       </c>
@@ -3608,7 +3628,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>484</v>
       </c>
@@ -3619,7 +3639,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>485</v>
       </c>
@@ -3630,7 +3650,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>486</v>
       </c>
@@ -3641,7 +3661,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>487</v>
       </c>
@@ -3652,7 +3672,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>488</v>
       </c>
@@ -3663,7 +3683,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>489</v>
       </c>
@@ -3674,7 +3694,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>490</v>
       </c>
@@ -3685,7 +3705,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>491</v>
       </c>
@@ -3696,7 +3716,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>492</v>
       </c>
@@ -3707,7 +3727,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>493</v>
       </c>
@@ -3718,7 +3738,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>494</v>
       </c>
@@ -3729,7 +3749,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>691</v>
       </c>
@@ -3740,7 +3760,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="16" t="s">
         <v>702</v>
       </c>
@@ -3751,7 +3771,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>495</v>
       </c>
@@ -3762,7 +3782,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>496</v>
       </c>
@@ -3773,7 +3793,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>497</v>
       </c>
@@ -3784,7 +3804,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>498</v>
       </c>
@@ -3795,7 +3815,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>499</v>
       </c>
@@ -3806,7 +3826,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>500</v>
       </c>
@@ -3817,7 +3837,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>501</v>
       </c>
@@ -3828,7 +3848,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>502</v>
       </c>
@@ -3839,7 +3859,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>503</v>
       </c>
@@ -3850,7 +3870,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>504</v>
       </c>
@@ -3861,7 +3881,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>505</v>
       </c>
@@ -3872,7 +3892,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>506</v>
       </c>
@@ -3883,7 +3903,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>507</v>
       </c>
@@ -3894,7 +3914,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>508</v>
       </c>
@@ -3905,7 +3925,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>509</v>
       </c>
@@ -3916,7 +3936,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>510</v>
       </c>
@@ -3927,7 +3947,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>511</v>
       </c>
@@ -3938,7 +3958,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>512</v>
       </c>
@@ -3949,7 +3969,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>513</v>
       </c>
@@ -3960,7 +3980,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>514</v>
       </c>
@@ -3971,7 +3991,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>515</v>
       </c>
@@ -3982,7 +4002,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>516</v>
       </c>
@@ -3993,7 +4013,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>517</v>
       </c>
@@ -4004,7 +4024,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>518</v>
       </c>
@@ -4015,7 +4035,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>519</v>
       </c>
@@ -4026,7 +4046,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>520</v>
       </c>
@@ -4037,7 +4057,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>521</v>
       </c>
@@ -4048,7 +4068,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>522</v>
       </c>
@@ -4059,7 +4079,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>523</v>
       </c>
@@ -4070,7 +4090,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>524</v>
       </c>
@@ -4081,7 +4101,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>525</v>
       </c>
@@ -4092,7 +4112,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>526</v>
       </c>
@@ -4103,7 +4123,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>527</v>
       </c>
@@ -4114,7 +4134,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>528</v>
       </c>
@@ -4125,7 +4145,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>529</v>
       </c>
@@ -4136,7 +4156,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>530</v>
       </c>
@@ -4147,7 +4167,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>531</v>
       </c>
@@ -4158,7 +4178,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>532</v>
       </c>
@@ -4169,7 +4189,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>533</v>
       </c>
@@ -4180,7 +4200,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>534</v>
       </c>
@@ -4191,7 +4211,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>535</v>
       </c>
@@ -4202,7 +4222,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>536</v>
       </c>
@@ -4213,7 +4233,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>537</v>
       </c>
@@ -4224,7 +4244,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>538</v>
       </c>
@@ -4235,7 +4255,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>539</v>
       </c>
@@ -4246,7 +4266,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>540</v>
       </c>
@@ -4257,7 +4277,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>541</v>
       </c>
@@ -4268,7 +4288,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>542</v>
       </c>
@@ -4279,7 +4299,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>543</v>
       </c>
@@ -4290,7 +4310,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>544</v>
       </c>
@@ -4301,7 +4321,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>545</v>
       </c>
@@ -4312,7 +4332,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>546</v>
       </c>
@@ -4323,7 +4343,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>547</v>
       </c>
@@ -4334,7 +4354,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>548</v>
       </c>
@@ -4345,7 +4365,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>549</v>
       </c>
@@ -4356,7 +4376,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>550</v>
       </c>
@@ -4367,7 +4387,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>551</v>
       </c>
@@ -4378,7 +4398,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>552</v>
       </c>
@@ -4389,7 +4409,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>553</v>
       </c>
@@ -4400,7 +4420,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>554</v>
       </c>
@@ -4411,7 +4431,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>555</v>
       </c>
@@ -4422,7 +4442,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>556</v>
       </c>
@@ -4433,7 +4453,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>557</v>
       </c>
@@ -4444,7 +4464,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>558</v>
       </c>
@@ -4455,7 +4475,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>559</v>
       </c>
@@ -4466,7 +4486,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>560</v>
       </c>
@@ -4477,7 +4497,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>561</v>
       </c>
@@ -4488,7 +4508,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>562</v>
       </c>
@@ -4499,7 +4519,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>563</v>
       </c>
@@ -4510,7 +4530,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>564</v>
       </c>
@@ -4521,7 +4541,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>565</v>
       </c>
@@ -4532,7 +4552,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>566</v>
       </c>
@@ -4543,7 +4563,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>567</v>
       </c>
@@ -4554,7 +4574,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>568</v>
       </c>
@@ -4565,7 +4585,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>569</v>
       </c>
@@ -4576,7 +4596,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>570</v>
       </c>
@@ -4587,7 +4607,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>571</v>
       </c>
@@ -4598,7 +4618,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>572</v>
       </c>
@@ -4609,7 +4629,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>573</v>
       </c>
@@ -4620,7 +4640,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>574</v>
       </c>
@@ -4631,7 +4651,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>575</v>
       </c>
@@ -4642,7 +4662,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>576</v>
       </c>
@@ -4653,7 +4673,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>577</v>
       </c>
@@ -4664,7 +4684,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>578</v>
       </c>
@@ -4675,7 +4695,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>579</v>
       </c>
@@ -4686,7 +4706,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>580</v>
       </c>
@@ -4697,7 +4717,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>581</v>
       </c>
@@ -4708,7 +4728,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>582</v>
       </c>
@@ -4719,7 +4739,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>583</v>
       </c>
@@ -4730,7 +4750,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>584</v>
       </c>
@@ -4741,7 +4761,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>585</v>
       </c>
@@ -4752,7 +4772,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>586</v>
       </c>
@@ -4763,7 +4783,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>587</v>
       </c>
@@ -4774,7 +4794,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>588</v>
       </c>
@@ -4785,7 +4805,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>589</v>
       </c>
@@ -4796,7 +4816,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>590</v>
       </c>
@@ -4807,7 +4827,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>658</v>
       </c>
@@ -4818,7 +4838,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>659</v>
       </c>
@@ -4829,7 +4849,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>660</v>
       </c>
@@ -4840,7 +4860,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>661</v>
       </c>
@@ -4851,7 +4871,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>662</v>
       </c>
@@ -4862,7 +4882,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>663</v>
       </c>
@@ -4873,7 +4893,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>664</v>
       </c>
@@ -4884,7 +4904,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>665</v>
       </c>
@@ -4895,7 +4915,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>666</v>
       </c>
@@ -4906,7 +4926,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>668</v>
       </c>
@@ -4917,7 +4937,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>591</v>
       </c>
@@ -4928,7 +4948,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>592</v>
       </c>
@@ -4939,7 +4959,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>593</v>
       </c>
@@ -4950,7 +4970,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>594</v>
       </c>
@@ -4961,7 +4981,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>667</v>
       </c>
@@ -4972,7 +4992,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>669</v>
       </c>
@@ -4983,7 +5003,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>670</v>
       </c>
@@ -4994,7 +5014,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>671</v>
       </c>
@@ -5005,7 +5025,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>672</v>
       </c>
@@ -5016,7 +5036,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>673</v>
       </c>
@@ -5027,7 +5047,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>674</v>
       </c>
@@ -5038,7 +5058,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>675</v>
       </c>
@@ -5049,7 +5069,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>676</v>
       </c>
@@ -5060,7 +5080,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>677</v>
       </c>
@@ -5071,7 +5091,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>595</v>
       </c>
@@ -5082,7 +5102,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>596</v>
       </c>
@@ -5093,7 +5113,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>678</v>
       </c>
@@ -5104,7 +5124,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>679</v>
       </c>
@@ -5115,7 +5135,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>597</v>
       </c>
@@ -5126,7 +5146,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>598</v>
       </c>
@@ -5137,7 +5157,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>599</v>
       </c>
@@ -5148,7 +5168,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>600</v>
       </c>
@@ -5159,7 +5179,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>601</v>
       </c>
@@ -5170,7 +5190,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>602</v>
       </c>
@@ -5181,7 +5201,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>603</v>
       </c>
@@ -5192,7 +5212,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>604</v>
       </c>
@@ -5203,7 +5223,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>605</v>
       </c>
@@ -5214,7 +5234,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>692</v>
       </c>
@@ -5225,7 +5245,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>693</v>
       </c>
@@ -5236,7 +5256,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>606</v>
       </c>
@@ -5247,7 +5267,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>607</v>
       </c>
@@ -5258,7 +5278,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>608</v>
       </c>
@@ -5269,7 +5289,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>609</v>
       </c>
@@ -5280,7 +5300,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>610</v>
       </c>
@@ -5291,7 +5311,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>611</v>
       </c>
@@ -5302,7 +5322,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>612</v>
       </c>
@@ -5313,7 +5333,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>613</v>
       </c>
@@ -5324,7 +5344,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>614</v>
       </c>
@@ -5335,7 +5355,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>615</v>
       </c>
@@ -5346,7 +5366,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>616</v>
       </c>
@@ -5357,7 +5377,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>617</v>
       </c>
@@ -5368,7 +5388,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>618</v>
       </c>
@@ -5379,7 +5399,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>619</v>
       </c>
@@ -5390,7 +5410,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>620</v>
       </c>
@@ -5401,7 +5421,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>621</v>
       </c>
@@ -5412,7 +5432,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>622</v>
       </c>
@@ -5423,7 +5443,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A246" s="15" t="s">
         <v>680</v>
       </c>
@@ -5434,7 +5454,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A247" s="15" t="s">
         <v>681</v>
       </c>
@@ -5445,7 +5465,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A248" s="15" t="s">
         <v>623</v>
       </c>
@@ -5456,7 +5476,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A249" s="15" t="s">
         <v>624</v>
       </c>
@@ -5467,7 +5487,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A250" s="15" t="s">
         <v>625</v>
       </c>
@@ -5478,7 +5498,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A251" s="15" t="s">
         <v>626</v>
       </c>
@@ -5489,7 +5509,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A252" s="15" t="s">
         <v>627</v>
       </c>
@@ -5500,7 +5520,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A253" s="15" t="s">
         <v>628</v>
       </c>
@@ -5511,7 +5531,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A254" s="15" t="s">
         <v>629</v>
       </c>
@@ -5522,7 +5542,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A255" s="15" t="s">
         <v>630</v>
       </c>
@@ -5533,7 +5553,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A256" s="15" t="s">
         <v>631</v>
       </c>
@@ -5544,7 +5564,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A257" s="15" t="s">
         <v>632</v>
       </c>
@@ -5555,7 +5575,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A258" s="15" t="s">
         <v>633</v>
       </c>
@@ -5566,7 +5586,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A259" s="15" t="s">
         <v>652</v>
       </c>
@@ -5577,7 +5597,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A260" s="15" t="s">
         <v>653</v>
       </c>
@@ -5588,7 +5608,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A261" s="15" t="s">
         <v>654</v>
       </c>
@@ -5599,7 +5619,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A262" s="15" t="s">
         <v>655</v>
       </c>
@@ -5610,7 +5630,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A263" s="15" t="s">
         <v>650</v>
       </c>
@@ -5621,7 +5641,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A264" s="15" t="s">
         <v>651</v>
       </c>
@@ -5632,7 +5652,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A265" s="16" t="s">
         <v>697</v>
       </c>
@@ -5643,7 +5663,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A266" s="16" t="s">
         <v>698</v>
       </c>
@@ -5654,7 +5674,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A267" s="16" t="s">
         <v>699</v>
       </c>
@@ -5665,7 +5685,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A268" s="16" t="s">
         <v>700</v>
       </c>
@@ -5676,7 +5696,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A269" s="16" t="s">
         <v>701</v>
       </c>
@@ -5687,7 +5707,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A270" s="15" t="s">
         <v>711</v>
       </c>
@@ -5696,6 +5716,39 @@
       </c>
       <c r="C270" s="3" t="s">
         <v>712</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A271" s="17" t="s">
+        <v>713</v>
+      </c>
+      <c r="B271" s="18" t="s">
+        <v>696</v>
+      </c>
+      <c r="C271" s="3" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A272" s="17" t="s">
+        <v>715</v>
+      </c>
+      <c r="B272" s="18" t="s">
+        <v>696</v>
+      </c>
+      <c r="C272" s="3" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A273" s="17" t="s">
+        <v>717</v>
+      </c>
+      <c r="B273" s="18" t="s">
+        <v>696</v>
+      </c>
+      <c r="C273" s="3" t="s">
+        <v>718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>